<commit_message>
Removing extra columns in the excel with aggregated data
</commit_message>
<xml_diff>
--- a/2026-ECMFA/results/aggregated_data.xlsx
+++ b/2026-ECMFA/results/aggregated_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\articles\2026\ECMFA.2026\LLM-model-assist\articles\ECMFA.2026\eval\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyectos\emf-kaizen-experiments\2026-ECMFA\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14F035A1-BD98-469D-9190-262D36C16CDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBA46F4D-C148-466D-A6E0-5AFB1360F4E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{5E534634-D184-43E0-8CE6-ACB8266C413F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{5E534634-D184-43E0-8CE6-ACB8266C413F}"/>
   </bookViews>
   <sheets>
     <sheet name="total-case-study" sheetId="1" r:id="rId1"/>
@@ -189,7 +189,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="40">
+  <borders count="37">
     <border>
       <left/>
       <right/>
@@ -562,43 +562,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -732,7 +695,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -797,22 +760,13 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -860,17 +814,17 @@
     <xf numFmtId="2" fontId="0" fillId="5" borderId="22" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="30" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="32" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="29" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -890,10 +844,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -902,8 +856,8 @@
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -925,7 +879,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -9123,34 +9077,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4289763A-AEE0-4D1C-8C8C-6D5A50C5DCA3}">
-  <dimension ref="A1:M30"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:K30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.1796875" customWidth="1"/>
-    <col min="2" max="13" width="6.26953125" customWidth="1"/>
+    <col min="1" max="1" width="16.140625" customWidth="1"/>
+    <col min="2" max="11" width="6.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="66" t="s">
+    <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="63" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="66" t="s">
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="63" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="67"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="66" t="s">
+      <c r="G1" s="64"/>
+      <c r="H1" s="65"/>
+      <c r="I1" s="63" t="s">
         <v>4</v>
       </c>
-      <c r="L1" s="67"/>
-      <c r="M1" s="68"/>
+      <c r="J1" s="64"/>
+      <c r="K1" s="65"/>
     </row>
-    <row r="2" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="1">
         <v>1</v>
       </c>
@@ -9163,48 +9115,40 @@
       <c r="E2" s="2">
         <v>4</v>
       </c>
-      <c r="F2" s="2">
-        <v>5</v>
-      </c>
-      <c r="G2" s="3">
-        <v>6</v>
-      </c>
-      <c r="H2" s="1">
+      <c r="F2" s="1">
         <v>1</v>
       </c>
-      <c r="I2" s="2">
+      <c r="G2" s="2">
         <v>2</v>
       </c>
-      <c r="J2" s="3">
+      <c r="H2" s="3">
         <v>3</v>
       </c>
-      <c r="K2" s="1">
+      <c r="I2" s="1">
         <v>1</v>
       </c>
-      <c r="L2" s="2">
+      <c r="J2" s="2">
         <v>2</v>
       </c>
-      <c r="M2" s="3">
+      <c r="K2" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="69" t="s">
+    <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="66" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="69"/>
-      <c r="D3" s="69"/>
-      <c r="E3" s="69"/>
-      <c r="F3" s="69"/>
-      <c r="G3" s="69"/>
-      <c r="H3" s="69"/>
-      <c r="I3" s="69"/>
-      <c r="J3" s="69"/>
-      <c r="K3" s="69"/>
-      <c r="L3" s="69"/>
-      <c r="M3" s="69"/>
+      <c r="C3" s="66"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="66"/>
+      <c r="F3" s="66"/>
+      <c r="G3" s="66"/>
+      <c r="H3" s="66"/>
+      <c r="I3" s="66"/>
+      <c r="J3" s="66"/>
+      <c r="K3" s="66"/>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>0</v>
       </c>
@@ -9220,36 +9164,30 @@
       <c r="E4" s="12">
         <v>0</v>
       </c>
-      <c r="F4" s="12">
+      <c r="F4" s="14">
+        <v>95.8</v>
+      </c>
+      <c r="G4" s="12">
         <v>0</v>
       </c>
-      <c r="G4" s="24">
+      <c r="H4" s="13">
+        <v>4.2</v>
+      </c>
+      <c r="I4" s="14">
         <v>0</v>
       </c>
-      <c r="H4" s="14">
+      <c r="J4" s="12">
+        <v>4.17</v>
+      </c>
+      <c r="K4" s="31">
         <v>95.8</v>
       </c>
-      <c r="I4" s="12">
-        <v>0</v>
-      </c>
-      <c r="J4" s="13">
-        <v>4.2</v>
-      </c>
-      <c r="K4" s="14">
-        <v>0</v>
-      </c>
-      <c r="L4" s="12">
-        <v>4.17</v>
-      </c>
-      <c r="M4" s="34">
-        <v>95.8</v>
-      </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="42">
+      <c r="B5" s="39">
         <v>100</v>
       </c>
       <c r="C5" s="16">
@@ -9261,32 +9199,26 @@
       <c r="E5" s="16">
         <v>0</v>
       </c>
-      <c r="F5" s="16">
+      <c r="F5" s="18">
+        <v>70.83</v>
+      </c>
+      <c r="G5" s="16">
+        <v>12.5</v>
+      </c>
+      <c r="H5" s="17">
+        <v>16.670000000000002</v>
+      </c>
+      <c r="I5" s="18">
         <v>0</v>
       </c>
-      <c r="G5" s="25">
-        <v>0</v>
-      </c>
-      <c r="H5" s="18">
-        <v>70.83</v>
-      </c>
-      <c r="I5" s="16">
-        <v>12.5</v>
-      </c>
-      <c r="J5" s="17">
-        <v>16.670000000000002</v>
-      </c>
-      <c r="K5" s="18">
-        <v>0</v>
-      </c>
-      <c r="L5" s="16">
+      <c r="J5" s="16">
         <v>4.17</v>
       </c>
-      <c r="M5" s="35">
+      <c r="K5" s="32">
         <v>95.8</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>2</v>
       </c>
@@ -9302,36 +9234,30 @@
       <c r="E6" s="16">
         <v>0</v>
       </c>
-      <c r="F6" s="16">
+      <c r="F6" s="18">
+        <v>87.5</v>
+      </c>
+      <c r="G6" s="16">
+        <v>8.33</v>
+      </c>
+      <c r="H6" s="17">
+        <v>4.17</v>
+      </c>
+      <c r="I6" s="18">
         <v>0</v>
       </c>
-      <c r="G6" s="25">
-        <v>0</v>
-      </c>
-      <c r="H6" s="18">
+      <c r="J6" s="16">
+        <v>12.5</v>
+      </c>
+      <c r="K6" s="17">
         <v>87.5</v>
       </c>
-      <c r="I6" s="16">
-        <v>8.33</v>
-      </c>
-      <c r="J6" s="17">
-        <v>4.17</v>
-      </c>
-      <c r="K6" s="18">
-        <v>0</v>
-      </c>
-      <c r="L6" s="16">
-        <v>12.5</v>
-      </c>
-      <c r="M6" s="17">
-        <v>87.5</v>
-      </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="42">
+      <c r="B7" s="39">
         <v>100</v>
       </c>
       <c r="C7" s="16">
@@ -9343,36 +9269,30 @@
       <c r="E7" s="16">
         <v>0</v>
       </c>
-      <c r="F7" s="16">
+      <c r="F7" s="18">
+        <v>79.16</v>
+      </c>
+      <c r="G7" s="16">
         <v>0</v>
       </c>
-      <c r="G7" s="25">
+      <c r="H7" s="17">
+        <v>20.83</v>
+      </c>
+      <c r="I7" s="18">
         <v>0</v>
       </c>
-      <c r="H7" s="18">
-        <v>79.16</v>
-      </c>
-      <c r="I7" s="16">
-        <v>0</v>
-      </c>
-      <c r="J7" s="17">
-        <v>20.83</v>
-      </c>
-      <c r="K7" s="18">
-        <v>0</v>
-      </c>
-      <c r="L7" s="16">
+      <c r="J7" s="16">
         <v>8.33</v>
       </c>
-      <c r="M7" s="17">
+      <c r="K7" s="17">
         <v>91.67</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="48" t="s">
+    <row r="8" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="44">
+      <c r="B8" s="41">
         <v>95.833333333333329</v>
       </c>
       <c r="C8" s="19">
@@ -9384,36 +9304,30 @@
       <c r="E8" s="19">
         <v>0</v>
       </c>
-      <c r="F8" s="19">
+      <c r="F8" s="27">
+        <v>87.5</v>
+      </c>
+      <c r="G8" s="28">
         <v>0</v>
       </c>
-      <c r="G8" s="26">
+      <c r="H8" s="29">
+        <v>12.5</v>
+      </c>
+      <c r="I8" s="20">
         <v>0</v>
       </c>
-      <c r="H8" s="30">
-        <v>87.5</v>
-      </c>
-      <c r="I8" s="31">
-        <v>0</v>
-      </c>
-      <c r="J8" s="32">
-        <v>12.5</v>
-      </c>
-      <c r="K8" s="20">
-        <v>0</v>
-      </c>
-      <c r="L8" s="19">
+      <c r="J8" s="19">
         <v>8.33</v>
       </c>
-      <c r="M8" s="36">
+      <c r="K8" s="33">
         <v>91.67</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="49" t="s">
+    <row r="9" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="33">
+      <c r="B9" s="30">
         <v>90.83</v>
       </c>
       <c r="C9" s="22">
@@ -9425,52 +9339,44 @@
       <c r="E9" s="22">
         <v>0</v>
       </c>
-      <c r="F9" s="22">
+      <c r="F9" s="24">
+        <v>84.17</v>
+      </c>
+      <c r="G9" s="25">
+        <v>4.17</v>
+      </c>
+      <c r="H9" s="26">
+        <v>11.67</v>
+      </c>
+      <c r="I9" s="21">
         <v>0</v>
       </c>
-      <c r="G9" s="23">
-        <v>0</v>
-      </c>
-      <c r="H9" s="27">
-        <v>84.17</v>
-      </c>
-      <c r="I9" s="28">
-        <v>4.17</v>
-      </c>
-      <c r="J9" s="29">
-        <v>11.67</v>
-      </c>
-      <c r="K9" s="21">
-        <v>0</v>
-      </c>
-      <c r="L9" s="22">
+      <c r="J9" s="22">
         <v>7.5</v>
       </c>
-      <c r="M9" s="23">
+      <c r="K9" s="23">
         <v>92.5</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B10" s="69" t="s">
+    <row r="10" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="66" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="69"/>
-      <c r="D10" s="69"/>
-      <c r="E10" s="69"/>
-      <c r="F10" s="69"/>
-      <c r="G10" s="69"/>
-      <c r="H10" s="69"/>
-      <c r="I10" s="69"/>
-      <c r="J10" s="69"/>
-      <c r="K10" s="69"/>
-      <c r="L10" s="69"/>
-      <c r="M10" s="69"/>
+      <c r="C10" s="66"/>
+      <c r="D10" s="66"/>
+      <c r="E10" s="66"/>
+      <c r="F10" s="66"/>
+      <c r="G10" s="66"/>
+      <c r="H10" s="66"/>
+      <c r="I10" s="66"/>
+      <c r="J10" s="66"/>
+      <c r="K10" s="66"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="41">
+      <c r="B11" s="38">
         <v>95.833333333333329</v>
       </c>
       <c r="C11" s="12">
@@ -9482,32 +9388,26 @@
       <c r="E11" s="12">
         <v>0</v>
       </c>
-      <c r="F11" s="12">
+      <c r="F11" s="14">
+        <v>95.83</v>
+      </c>
+      <c r="G11" s="12">
         <v>0</v>
       </c>
-      <c r="G11" s="13">
+      <c r="H11" s="13">
+        <v>4.17</v>
+      </c>
+      <c r="I11" s="11">
         <v>0</v>
       </c>
-      <c r="H11" s="14">
-        <v>95.83</v>
-      </c>
-      <c r="I11" s="12">
-        <v>0</v>
-      </c>
-      <c r="J11" s="13">
-        <v>4.17</v>
-      </c>
-      <c r="K11" s="11">
-        <v>0</v>
-      </c>
-      <c r="L11" s="12">
+      <c r="J11" s="12">
         <v>33.33</v>
       </c>
-      <c r="M11" s="13">
+      <c r="K11" s="13">
         <v>66.67</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>1</v>
       </c>
@@ -9523,32 +9423,26 @@
       <c r="E12" s="16">
         <v>0</v>
       </c>
-      <c r="F12" s="16">
+      <c r="F12" s="40">
+        <v>100</v>
+      </c>
+      <c r="G12" s="16">
         <v>0</v>
       </c>
-      <c r="G12" s="17">
+      <c r="H12" s="17">
         <v>0</v>
       </c>
-      <c r="H12" s="43">
-        <v>100</v>
-      </c>
-      <c r="I12" s="16">
+      <c r="I12" s="15">
         <v>0</v>
       </c>
-      <c r="J12" s="17">
-        <v>0</v>
-      </c>
-      <c r="K12" s="15">
-        <v>0</v>
-      </c>
-      <c r="L12" s="16">
+      <c r="J12" s="16">
         <v>8.33</v>
       </c>
-      <c r="M12" s="17">
+      <c r="K12" s="17">
         <v>91.67</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>2</v>
       </c>
@@ -9564,36 +9458,30 @@
       <c r="E13" s="16">
         <v>0</v>
       </c>
-      <c r="F13" s="16">
+      <c r="F13" s="40">
+        <v>100</v>
+      </c>
+      <c r="G13" s="16">
         <v>0</v>
       </c>
-      <c r="G13" s="17">
+      <c r="H13" s="17">
         <v>0</v>
       </c>
-      <c r="H13" s="43">
-        <v>100</v>
-      </c>
-      <c r="I13" s="16">
+      <c r="I13" s="15">
         <v>0</v>
       </c>
-      <c r="J13" s="17">
-        <v>0</v>
-      </c>
-      <c r="K13" s="15">
-        <v>0</v>
-      </c>
-      <c r="L13" s="16">
+      <c r="J13" s="16">
         <v>4.17</v>
       </c>
-      <c r="M13" s="35">
+      <c r="K13" s="32">
         <v>95.83</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B14" s="43">
+      <c r="B14" s="40">
         <v>100</v>
       </c>
       <c r="C14" s="16">
@@ -9605,32 +9493,26 @@
       <c r="E14" s="16">
         <v>0</v>
       </c>
-      <c r="F14" s="16">
+      <c r="F14" s="40">
+        <v>100</v>
+      </c>
+      <c r="G14" s="16">
         <v>0</v>
       </c>
-      <c r="G14" s="17">
+      <c r="H14" s="17">
         <v>0</v>
       </c>
-      <c r="H14" s="43">
-        <v>100</v>
-      </c>
-      <c r="I14" s="16">
+      <c r="I14" s="15">
         <v>0</v>
       </c>
-      <c r="J14" s="17">
-        <v>0</v>
-      </c>
-      <c r="K14" s="15">
-        <v>0</v>
-      </c>
-      <c r="L14" s="16">
+      <c r="J14" s="16">
         <v>4.17</v>
       </c>
-      <c r="M14" s="35">
+      <c r="K14" s="32">
         <v>95.83</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>3</v>
       </c>
@@ -9646,32 +9528,26 @@
       <c r="E15" s="16">
         <v>0</v>
       </c>
-      <c r="F15" s="16">
+      <c r="F15" s="27">
+        <v>87.5</v>
+      </c>
+      <c r="G15" s="28">
         <v>0</v>
       </c>
-      <c r="G15" s="17">
+      <c r="H15" s="29">
+        <v>12.5</v>
+      </c>
+      <c r="I15" s="15">
         <v>0</v>
       </c>
-      <c r="H15" s="30">
-        <v>87.5</v>
-      </c>
-      <c r="I15" s="31">
-        <v>0</v>
-      </c>
-      <c r="J15" s="32">
-        <v>12.5</v>
-      </c>
-      <c r="K15" s="15">
-        <v>0</v>
-      </c>
-      <c r="L15" s="16">
+      <c r="J15" s="16">
         <v>8.33</v>
       </c>
-      <c r="M15" s="35">
+      <c r="K15" s="32">
         <v>91.67</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
         <v>7</v>
       </c>
@@ -9687,48 +9563,40 @@
       <c r="E16" s="7">
         <v>0</v>
       </c>
-      <c r="F16" s="7">
+      <c r="F16" s="9">
+        <v>96.67</v>
+      </c>
+      <c r="G16" s="7">
         <v>0</v>
       </c>
-      <c r="G16" s="8">
+      <c r="H16" s="8">
+        <v>3.33</v>
+      </c>
+      <c r="I16" s="6">
         <v>0</v>
       </c>
-      <c r="H16" s="9">
-        <v>96.67</v>
-      </c>
-      <c r="I16" s="7">
-        <v>0</v>
-      </c>
-      <c r="J16" s="8">
-        <v>3.33</v>
-      </c>
-      <c r="K16" s="6">
-        <v>0</v>
-      </c>
-      <c r="L16" s="7">
+      <c r="J16" s="7">
         <v>11.67</v>
       </c>
-      <c r="M16" s="8">
+      <c r="K16" s="8">
         <v>88.33</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B17" s="69" t="s">
+    <row r="17" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="C17" s="69"/>
-      <c r="D17" s="69"/>
-      <c r="E17" s="69"/>
-      <c r="F17" s="69"/>
-      <c r="G17" s="69"/>
-      <c r="H17" s="69"/>
-      <c r="I17" s="69"/>
-      <c r="J17" s="69"/>
-      <c r="K17" s="69"/>
-      <c r="L17" s="69"/>
-      <c r="M17" s="69"/>
+      <c r="C17" s="66"/>
+      <c r="D17" s="66"/>
+      <c r="E17" s="66"/>
+      <c r="F17" s="66"/>
+      <c r="G17" s="66"/>
+      <c r="H17" s="66"/>
+      <c r="I17" s="66"/>
+      <c r="J17" s="66"/>
+      <c r="K17" s="66"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>0</v>
       </c>
@@ -9742,34 +9610,28 @@
         <v>8.3333333333333339</v>
       </c>
       <c r="E18" s="12">
+        <v>12.5</v>
+      </c>
+      <c r="F18" s="38">
+        <v>100</v>
+      </c>
+      <c r="G18" s="12">
         <v>0</v>
       </c>
-      <c r="F18" s="12">
+      <c r="H18" s="13">
+        <v>0</v>
+      </c>
+      <c r="I18" s="11">
         <v>12.5</v>
       </c>
-      <c r="G18" s="13">
-        <v>0</v>
-      </c>
-      <c r="H18" s="41">
-        <v>100</v>
-      </c>
-      <c r="I18" s="12">
-        <v>0</v>
-      </c>
-      <c r="J18" s="13">
-        <v>0</v>
-      </c>
-      <c r="K18" s="11">
-        <v>12.5</v>
-      </c>
-      <c r="L18" s="12">
+      <c r="J18" s="12">
         <v>25</v>
       </c>
-      <c r="M18" s="13">
+      <c r="K18" s="13">
         <v>62.5</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>1</v>
       </c>
@@ -9783,34 +9645,28 @@
         <v>0</v>
       </c>
       <c r="E19" s="16">
-        <v>0</v>
-      </c>
-      <c r="F19" s="16">
         <v>4.166666666666667</v>
       </c>
-      <c r="G19" s="17">
-        <v>0</v>
-      </c>
-      <c r="H19" s="18">
+      <c r="F19" s="18">
         <v>91.3</v>
       </c>
-      <c r="I19" s="16">
+      <c r="G19" s="16">
         <v>4.34</v>
       </c>
-      <c r="J19" s="17">
+      <c r="H19" s="17">
         <v>4.34</v>
       </c>
-      <c r="K19" s="15">
+      <c r="I19" s="15">
         <v>4.17</v>
       </c>
-      <c r="L19" s="16">
+      <c r="J19" s="16">
         <v>20.83</v>
       </c>
-      <c r="M19" s="17">
+      <c r="K19" s="17">
         <v>75</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>2</v>
       </c>
@@ -9824,34 +9680,28 @@
         <v>0</v>
       </c>
       <c r="E20" s="16">
+        <v>12.5</v>
+      </c>
+      <c r="F20" s="18">
+        <v>90.47</v>
+      </c>
+      <c r="G20" s="16">
+        <v>9.52</v>
+      </c>
+      <c r="H20" s="17">
         <v>0</v>
       </c>
-      <c r="F20" s="16">
+      <c r="I20" s="15">
         <v>12.5</v>
       </c>
-      <c r="G20" s="17">
-        <v>0</v>
-      </c>
-      <c r="H20" s="18">
-        <v>90.47</v>
-      </c>
-      <c r="I20" s="16">
-        <v>9.52</v>
-      </c>
-      <c r="J20" s="17">
-        <v>0</v>
-      </c>
-      <c r="K20" s="15">
-        <v>12.5</v>
-      </c>
-      <c r="L20" s="16">
+      <c r="J20" s="16">
         <v>45.83</v>
       </c>
-      <c r="M20" s="17">
+      <c r="K20" s="17">
         <v>41.67</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>10</v>
       </c>
@@ -9865,34 +9715,28 @@
         <v>0</v>
       </c>
       <c r="E21" s="16">
+        <v>12.5</v>
+      </c>
+      <c r="F21" s="18">
+        <v>95.24</v>
+      </c>
+      <c r="G21" s="16">
+        <v>4.76</v>
+      </c>
+      <c r="H21" s="17">
         <v>0</v>
       </c>
-      <c r="F21" s="16">
-        <v>12.5</v>
-      </c>
-      <c r="G21" s="17">
-        <v>0</v>
-      </c>
-      <c r="H21" s="18">
-        <v>95.24</v>
-      </c>
-      <c r="I21" s="16">
-        <v>4.76</v>
-      </c>
-      <c r="J21" s="17">
-        <v>0</v>
-      </c>
-      <c r="K21" s="15">
+      <c r="I21" s="15">
         <v>16.670000000000002</v>
       </c>
-      <c r="L21" s="16">
+      <c r="J21" s="16">
         <v>20.83</v>
       </c>
-      <c r="M21" s="17">
+      <c r="K21" s="17">
         <v>62.5</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>3</v>
       </c>
@@ -9906,91 +9750,77 @@
         <v>12.5</v>
       </c>
       <c r="E22" s="16">
+        <v>16.666666666666668</v>
+      </c>
+      <c r="F22" s="40">
+        <v>90</v>
+      </c>
+      <c r="G22" s="16">
+        <v>10</v>
+      </c>
+      <c r="H22" s="17">
         <v>0</v>
       </c>
-      <c r="F22" s="16">
-        <v>16.666666666666668</v>
-      </c>
-      <c r="G22" s="17">
-        <v>0</v>
-      </c>
-      <c r="H22" s="43">
-        <v>90</v>
-      </c>
-      <c r="I22" s="16">
-        <v>10</v>
-      </c>
-      <c r="J22" s="17">
-        <v>0</v>
-      </c>
-      <c r="K22" s="15">
+      <c r="I22" s="15">
         <v>20.83</v>
       </c>
-      <c r="L22" s="16">
+      <c r="J22" s="16">
         <v>25</v>
       </c>
-      <c r="M22" s="17">
+      <c r="K22" s="17">
         <v>54.17</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="B23" s="40">
+      <c r="B23" s="37">
         <v>84.17</v>
       </c>
-      <c r="C23" s="38">
+      <c r="C23" s="35">
         <v>0</v>
       </c>
-      <c r="D23" s="38">
+      <c r="D23" s="35">
         <v>4.17</v>
       </c>
-      <c r="E23" s="38">
-        <v>0</v>
-      </c>
-      <c r="F23" s="38">
+      <c r="E23" s="35">
         <v>11.67</v>
       </c>
-      <c r="G23" s="39">
-        <v>0</v>
-      </c>
-      <c r="H23" s="40">
+      <c r="F23" s="37">
         <v>93.4</v>
       </c>
-      <c r="I23" s="38">
+      <c r="G23" s="35">
         <v>5.66</v>
       </c>
-      <c r="J23" s="39">
+      <c r="H23" s="36">
         <v>0.95</v>
       </c>
-      <c r="K23" s="37">
+      <c r="I23" s="34">
         <v>13.33</v>
       </c>
-      <c r="L23" s="38">
+      <c r="J23" s="35">
         <v>27.5</v>
       </c>
-      <c r="M23" s="39">
+      <c r="K23" s="36">
         <v>59.17</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B24" s="69" t="s">
+    <row r="24" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="C24" s="69"/>
-      <c r="D24" s="69"/>
-      <c r="E24" s="69"/>
-      <c r="F24" s="69"/>
-      <c r="G24" s="69"/>
-      <c r="H24" s="69"/>
-      <c r="I24" s="69"/>
-      <c r="J24" s="69"/>
-      <c r="K24" s="69"/>
-      <c r="L24" s="69"/>
-      <c r="M24" s="69"/>
+      <c r="C24" s="66"/>
+      <c r="D24" s="66"/>
+      <c r="E24" s="66"/>
+      <c r="F24" s="66"/>
+      <c r="G24" s="66"/>
+      <c r="H24" s="66"/>
+      <c r="I24" s="66"/>
+      <c r="J24" s="66"/>
+      <c r="K24" s="66"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>0</v>
       </c>
@@ -10006,32 +9836,26 @@
       <c r="E25" s="12">
         <v>0</v>
       </c>
-      <c r="F25" s="12">
+      <c r="F25" s="38">
+        <v>100</v>
+      </c>
+      <c r="G25" s="12">
         <v>0</v>
       </c>
-      <c r="G25" s="24">
+      <c r="H25" s="13">
         <v>0</v>
       </c>
-      <c r="H25" s="41">
-        <v>100</v>
-      </c>
-      <c r="I25" s="12">
-        <v>0</v>
-      </c>
-      <c r="J25" s="13">
-        <v>0</v>
-      </c>
-      <c r="K25" s="11">
+      <c r="I25" s="11">
         <v>4.17</v>
       </c>
-      <c r="L25" s="12">
+      <c r="J25" s="12">
         <v>37.5</v>
       </c>
-      <c r="M25" s="13">
+      <c r="K25" s="13">
         <v>58.33</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>1</v>
       </c>
@@ -10047,36 +9871,30 @@
       <c r="E26" s="16">
         <v>0</v>
       </c>
-      <c r="F26" s="16">
+      <c r="F26" s="40">
+        <v>100</v>
+      </c>
+      <c r="G26" s="16">
         <v>0</v>
       </c>
-      <c r="G26" s="25">
+      <c r="H26" s="17">
         <v>0</v>
       </c>
-      <c r="H26" s="43">
-        <v>100</v>
-      </c>
-      <c r="I26" s="16">
+      <c r="I26" s="15">
         <v>0</v>
       </c>
-      <c r="J26" s="17">
-        <v>0</v>
-      </c>
-      <c r="K26" s="15">
-        <v>0</v>
-      </c>
-      <c r="L26" s="16">
+      <c r="J26" s="16">
         <v>12.5</v>
       </c>
-      <c r="M26" s="17">
+      <c r="K26" s="17">
         <v>87.5</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B27" s="43">
+      <c r="B27" s="40">
         <v>91.666666666666671</v>
       </c>
       <c r="C27" s="16">
@@ -10088,32 +9906,26 @@
       <c r="E27" s="16">
         <v>0</v>
       </c>
-      <c r="F27" s="16">
+      <c r="F27" s="40">
+        <v>100</v>
+      </c>
+      <c r="G27" s="16">
         <v>0</v>
       </c>
-      <c r="G27" s="25">
+      <c r="H27" s="17">
         <v>0</v>
       </c>
-      <c r="H27" s="43">
-        <v>100</v>
-      </c>
-      <c r="I27" s="16">
-        <v>0</v>
-      </c>
-      <c r="J27" s="17">
-        <v>0</v>
-      </c>
-      <c r="K27" s="15">
+      <c r="I27" s="15">
         <v>8.33</v>
       </c>
-      <c r="L27" s="16">
+      <c r="J27" s="16">
         <v>25</v>
       </c>
-      <c r="M27" s="17">
+      <c r="K27" s="17">
         <v>66.67</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>10</v>
       </c>
@@ -10129,32 +9941,26 @@
       <c r="E28" s="16">
         <v>0</v>
       </c>
-      <c r="F28" s="16">
+      <c r="F28" s="40">
+        <v>100</v>
+      </c>
+      <c r="G28" s="16">
         <v>0</v>
       </c>
-      <c r="G28" s="25">
+      <c r="H28" s="17">
         <v>0</v>
       </c>
-      <c r="H28" s="43">
-        <v>100</v>
-      </c>
-      <c r="I28" s="16">
-        <v>0</v>
-      </c>
-      <c r="J28" s="17">
-        <v>0</v>
-      </c>
-      <c r="K28" s="15">
+      <c r="I28" s="15">
         <v>16.670000000000002</v>
       </c>
-      <c r="L28" s="16">
+      <c r="J28" s="16">
         <v>25</v>
       </c>
-      <c r="M28" s="17">
+      <c r="K28" s="17">
         <v>58.33</v>
       </c>
     </row>
-    <row r="29" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>3</v>
       </c>
@@ -10170,81 +9976,69 @@
       <c r="E29" s="16">
         <v>0</v>
       </c>
-      <c r="F29" s="16">
+      <c r="F29" s="27">
+        <v>83.33</v>
+      </c>
+      <c r="G29" s="28">
         <v>0</v>
       </c>
-      <c r="G29" s="25">
-        <v>0</v>
-      </c>
-      <c r="H29" s="30">
-        <v>83.33</v>
-      </c>
-      <c r="I29" s="31">
-        <v>0</v>
-      </c>
-      <c r="J29" s="32">
+      <c r="H29" s="29">
         <v>16.670000000000002</v>
       </c>
-      <c r="K29" s="15">
+      <c r="I29" s="15">
         <v>4.17</v>
       </c>
-      <c r="L29" s="16">
+      <c r="J29" s="16">
         <v>25</v>
       </c>
-      <c r="M29" s="17">
+      <c r="K29" s="17">
         <v>70.83</v>
       </c>
     </row>
-    <row r="30" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="B30" s="40">
+      <c r="B30" s="37">
         <v>82.5</v>
       </c>
-      <c r="C30" s="38">
+      <c r="C30" s="35">
         <v>0.83</v>
       </c>
-      <c r="D30" s="38">
+      <c r="D30" s="35">
         <v>16.670000000000002</v>
       </c>
-      <c r="E30" s="38">
+      <c r="E30" s="35">
         <v>0</v>
       </c>
-      <c r="F30" s="38">
+      <c r="F30" s="42">
+        <v>96.67</v>
+      </c>
+      <c r="G30" s="43">
         <v>0</v>
       </c>
-      <c r="G30" s="39">
-        <v>0</v>
-      </c>
-      <c r="H30" s="45">
-        <v>96.67</v>
-      </c>
-      <c r="I30" s="46">
-        <v>0</v>
-      </c>
-      <c r="J30" s="47">
+      <c r="H30" s="44">
         <v>3.33</v>
       </c>
-      <c r="K30" s="37">
+      <c r="I30" s="34">
         <v>6.67</v>
       </c>
-      <c r="L30" s="38">
+      <c r="J30" s="35">
         <v>25</v>
       </c>
-      <c r="M30" s="39">
+      <c r="K30" s="36">
         <v>68.33</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="K1:M1"/>
-    <mergeCell ref="B3:M3"/>
-    <mergeCell ref="B10:M10"/>
-    <mergeCell ref="B17:M17"/>
-    <mergeCell ref="B24:M24"/>
-    <mergeCell ref="B1:G1"/>
-    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="B10:K10"/>
+    <mergeCell ref="B17:K17"/>
+    <mergeCell ref="B24:K24"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="F1:H1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10253,265 +10047,265 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51FA7C9A-54D9-4D41-810F-DB751F1B4B1E}">
   <dimension ref="A1:E18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.7265625" style="53" customWidth="1"/>
-    <col min="2" max="5" width="15.1796875" customWidth="1"/>
+    <col min="1" max="1" width="19.7109375" style="50" customWidth="1"/>
+    <col min="2" max="5" width="15.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
+    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
     </row>
-    <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="50" t="s">
+    <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="51" t="s">
+      <c r="C2" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="51" t="s">
+      <c r="D2" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="51" t="s">
+      <c r="E2" s="48" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3"/>
-      <c r="B3" s="70" t="s">
+      <c r="B3" s="67" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="70"/>
-      <c r="D3" s="70"/>
-      <c r="E3" s="70"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
     </row>
-    <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="54" t="s">
+    <row r="4" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="55">
+      <c r="B4" s="52">
         <v>0</v>
       </c>
-      <c r="C4" s="55">
+      <c r="C4" s="52">
         <v>0</v>
       </c>
-      <c r="D4" s="55">
+      <c r="D4" s="52">
         <v>0</v>
       </c>
-      <c r="E4" s="55">
+      <c r="E4" s="52">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="52" t="s">
+    <row r="5" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="55">
+      <c r="B5" s="52">
         <v>3.3333333333333335</v>
       </c>
-      <c r="C5" s="55">
+      <c r="C5" s="52">
         <v>6.666666666666667</v>
       </c>
-      <c r="D5" s="55">
+      <c r="D5" s="52">
         <v>0</v>
       </c>
-      <c r="E5" s="55">
+      <c r="E5" s="52">
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="52" t="s">
+    <row r="6" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="55">
+      <c r="B6" s="52">
         <v>96.666666666666671</v>
       </c>
-      <c r="C6" s="55">
+      <c r="C6" s="52">
         <v>93.333333333333329</v>
       </c>
-      <c r="D6" s="55">
+      <c r="D6" s="52">
         <v>100</v>
       </c>
-      <c r="E6" s="55">
+      <c r="E6" s="52">
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="70" t="s">
+    <row r="7" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="67" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="70"/>
-      <c r="D7" s="70"/>
-      <c r="E7" s="70"/>
+      <c r="C7" s="67"/>
+      <c r="D7" s="67"/>
+      <c r="E7" s="67"/>
     </row>
-    <row r="8" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="54" t="s">
+    <row r="8" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="55">
+      <c r="B8" s="52">
         <v>0</v>
       </c>
-      <c r="C8" s="55">
+      <c r="C8" s="52">
         <v>0</v>
       </c>
-      <c r="D8" s="55">
+      <c r="D8" s="52">
         <v>0</v>
       </c>
-      <c r="E8" s="55">
+      <c r="E8" s="52">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="52" t="s">
+    <row r="9" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="55">
+      <c r="B9" s="52">
         <v>0</v>
       </c>
-      <c r="C9" s="55">
+      <c r="C9" s="52">
         <v>16.666666666666668</v>
       </c>
-      <c r="D9" s="55">
+      <c r="D9" s="52">
         <v>13.333333333333334</v>
       </c>
-      <c r="E9" s="55">
+      <c r="E9" s="52">
         <v>16.666666666666668</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="52" t="s">
+    <row r="10" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="55">
+      <c r="B10" s="52">
         <v>100</v>
       </c>
-      <c r="C10" s="55">
+      <c r="C10" s="52">
         <v>83.333333333333329</v>
       </c>
-      <c r="D10" s="55">
+      <c r="D10" s="52">
         <v>86.666666666666671</v>
       </c>
-      <c r="E10" s="55">
+      <c r="E10" s="52">
         <v>83.333333333333329</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B11" s="70" t="s">
+    <row r="11" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="67" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="70"/>
-      <c r="D11" s="70"/>
-      <c r="E11" s="70"/>
+      <c r="C11" s="67"/>
+      <c r="D11" s="67"/>
+      <c r="E11" s="67"/>
     </row>
-    <row r="12" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="54" t="s">
+    <row r="12" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="55">
+      <c r="B12" s="52">
         <v>0</v>
       </c>
-      <c r="C12" s="55">
+      <c r="C12" s="52">
         <v>46.666666666666664</v>
       </c>
-      <c r="D12" s="55">
+      <c r="D12" s="52">
         <v>0</v>
       </c>
-      <c r="E12" s="55">
+      <c r="E12" s="52">
         <v>6.666666666666667</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="52" t="s">
+    <row r="13" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="55">
+      <c r="B13" s="52">
         <v>13.333333333333334</v>
       </c>
-      <c r="C13" s="55">
+      <c r="C13" s="52">
         <v>16.666666666666668</v>
       </c>
-      <c r="D13" s="55">
+      <c r="D13" s="52">
         <v>30</v>
       </c>
-      <c r="E13" s="55">
+      <c r="E13" s="52">
         <v>50</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="52" t="s">
+    <row r="14" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="55">
+      <c r="B14" s="52">
         <v>86.666666666666671</v>
       </c>
-      <c r="C14" s="55">
+      <c r="C14" s="52">
         <v>36.666666666666664</v>
       </c>
-      <c r="D14" s="55">
+      <c r="D14" s="52">
         <v>70</v>
       </c>
-      <c r="E14" s="55">
+      <c r="E14" s="52">
         <v>43.333333333333336</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B15" s="70" t="s">
+    <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="67" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="70"/>
-      <c r="D15" s="70"/>
-      <c r="E15" s="70"/>
+      <c r="C15" s="67"/>
+      <c r="D15" s="67"/>
+      <c r="E15" s="67"/>
     </row>
-    <row r="16" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="54" t="s">
+    <row r="16" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="55">
+      <c r="B16" s="52">
         <v>0</v>
       </c>
-      <c r="C16" s="55">
+      <c r="C16" s="52">
         <v>3.3333333333333335</v>
       </c>
-      <c r="D16" s="55">
+      <c r="D16" s="52">
         <v>6.666666666666667</v>
       </c>
-      <c r="E16" s="55">
+      <c r="E16" s="52">
         <v>16.666666666666668</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="52" t="s">
+    <row r="17" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="55">
+      <c r="B17" s="52">
         <v>13.333333333333334</v>
       </c>
-      <c r="C17" s="55">
+      <c r="C17" s="52">
         <v>13.333333333333334</v>
       </c>
-      <c r="D17" s="55">
+      <c r="D17" s="52">
         <v>33.333333333333336</v>
       </c>
-      <c r="E17" s="55">
+      <c r="E17" s="52">
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="52" t="s">
+    <row r="18" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="55">
+      <c r="B18" s="52">
         <v>86.666666666666671</v>
       </c>
-      <c r="C18" s="55">
+      <c r="C18" s="52">
         <v>83.333333333333329</v>
       </c>
-      <c r="D18" s="55">
+      <c r="D18" s="52">
         <v>60</v>
       </c>
-      <c r="E18" s="55">
+      <c r="E18" s="52">
         <v>43.333333333333336</v>
       </c>
     </row>
@@ -10531,106 +10325,106 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{348E115E-0FDE-4281-B378-3CA6BE68DB69}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.1796875" customWidth="1"/>
+    <col min="1" max="1" width="19.140625" customWidth="1"/>
     <col min="2" max="5" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B1" s="57" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B1" s="54" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="58" t="s">
+      <c r="C1" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="58" t="s">
+      <c r="D1" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="58" t="s">
+      <c r="E1" s="55" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="58" t="s">
+      <c r="F1" s="55" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="59">
+      <c r="B2" s="56">
         <v>6.2333333333333343</v>
       </c>
-      <c r="C2" s="59">
+      <c r="C2" s="56">
         <v>10.6</v>
       </c>
-      <c r="D2" s="59">
+      <c r="D2" s="56">
         <v>7.2333333333333325</v>
       </c>
-      <c r="E2" s="59">
+      <c r="E2" s="56">
         <v>21.233333333333334</v>
       </c>
-      <c r="F2" s="60">
+      <c r="F2" s="57">
         <v>11.291666666666666</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="59">
+      <c r="B3" s="56">
         <v>5.8999999999999995</v>
       </c>
-      <c r="C3" s="59">
+      <c r="C3" s="56">
         <v>10.7</v>
       </c>
-      <c r="D3" s="59">
+      <c r="D3" s="56">
         <v>5.0999999999999996</v>
       </c>
-      <c r="E3" s="59">
+      <c r="E3" s="56">
         <v>14.7</v>
       </c>
-      <c r="F3" s="60">
+      <c r="F3" s="57">
         <v>9.0583333333333336</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="59">
+      <c r="B4" s="56">
         <v>6.3000000000000007</v>
       </c>
-      <c r="C4" s="59">
+      <c r="C4" s="56">
         <v>3.7666666666666666</v>
       </c>
-      <c r="D4" s="59">
+      <c r="D4" s="56">
         <v>4.8666666666666663</v>
       </c>
-      <c r="E4" s="59">
+      <c r="E4" s="56">
         <v>8.1000000000000014</v>
       </c>
-      <c r="F4" s="60">
+      <c r="F4" s="57">
         <v>5.7333333333333334</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="59">
+      <c r="B5" s="56">
         <v>6.1666666666666661</v>
       </c>
-      <c r="C5" s="59">
+      <c r="C5" s="56">
         <v>9.966666666666665</v>
       </c>
-      <c r="D5" s="59">
+      <c r="D5" s="56">
         <v>4.5999999999999996</v>
       </c>
-      <c r="E5" s="59">
+      <c r="E5" s="56">
         <v>16.666666666666664</v>
       </c>
-      <c r="F5" s="60">
+      <c r="F5" s="57">
         <v>9.3249999999999993</v>
       </c>
     </row>
@@ -10643,106 +10437,106 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8440021D-2FC0-4232-9233-78C91580E9F6}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.1796875" customWidth="1"/>
+    <col min="1" max="1" width="19.140625" customWidth="1"/>
     <col min="2" max="5" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B1" s="57" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B1" s="54" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="58" t="s">
+      <c r="C1" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="58" t="s">
+      <c r="D1" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="58" t="s">
+      <c r="E1" s="55" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="58" t="s">
+      <c r="F1" s="55" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="59">
+      <c r="B2" s="56">
         <v>7.0333333333333332</v>
       </c>
-      <c r="C2" s="59">
+      <c r="C2" s="56">
         <v>10.633333333333333</v>
       </c>
-      <c r="D2" s="59">
+      <c r="D2" s="56">
         <v>7.4</v>
       </c>
-      <c r="E2" s="59">
+      <c r="E2" s="56">
         <v>23.1</v>
       </c>
-      <c r="F2" s="60">
+      <c r="F2" s="57">
         <v>12.008333333333333</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="59">
+      <c r="B3" s="56">
         <v>6</v>
       </c>
-      <c r="C3" s="59">
+      <c r="C3" s="56">
         <v>10.733333333333333</v>
       </c>
-      <c r="D3" s="59">
+      <c r="D3" s="56">
         <v>5.0999999999999996</v>
       </c>
-      <c r="E3" s="59">
+      <c r="E3" s="56">
         <v>14.7</v>
       </c>
-      <c r="F3" s="60">
+      <c r="F3" s="57">
         <v>9.0916666666666668</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="59">
+      <c r="B4" s="56">
         <v>6.3666666666666671</v>
       </c>
-      <c r="C4" s="59">
+      <c r="C4" s="56">
         <v>4.9666666666666668</v>
       </c>
-      <c r="D4" s="59">
+      <c r="D4" s="56">
         <v>4.8666666666666663</v>
       </c>
-      <c r="E4" s="59">
+      <c r="E4" s="56">
         <v>8.2666666666666675</v>
       </c>
-      <c r="F4" s="60">
+      <c r="F4" s="57">
         <v>6.0916666666666668</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="59">
+      <c r="B5" s="56">
         <v>6.2</v>
       </c>
-      <c r="C5" s="59">
+      <c r="C5" s="56">
         <v>10.166666666666666</v>
       </c>
-      <c r="D5" s="59">
+      <c r="D5" s="56">
         <v>4.9000000000000004</v>
       </c>
-      <c r="E5" s="59">
+      <c r="E5" s="56">
         <v>16.899999999999999</v>
       </c>
-      <c r="F5" s="60">
+      <c r="F5" s="57">
         <v>9.5166666666666675</v>
       </c>
     </row>
@@ -10755,37 +10549,37 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CAFDAB1-E659-4A34-ACEA-C7F1FCCC29AD}">
   <dimension ref="A1:H5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.1796875" customWidth="1"/>
-    <col min="2" max="8" width="10.7265625" style="56" customWidth="1"/>
+    <col min="1" max="1" width="17.140625" customWidth="1"/>
+    <col min="2" max="8" width="10.7109375" style="53" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="63" t="s">
+    <row r="1" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="63" t="s">
+      <c r="C1" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="63" t="s">
+      <c r="D1" s="60" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="63" t="s">
+      <c r="E1" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="65" t="s">
+      <c r="F1" s="62" t="s">
         <v>27</v>
       </c>
-      <c r="G1" s="63" t="s">
+      <c r="G1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="63" t="s">
+      <c r="H1" s="60" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" s="61" t="s">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="58" t="s">
         <v>26</v>
       </c>
       <c r="B2" s="16">
@@ -10800,18 +10594,18 @@
       <c r="E2" s="16">
         <v>61.1</v>
       </c>
-      <c r="F2" s="64">
+      <c r="F2" s="61">
         <v>31.105</v>
       </c>
-      <c r="G2" s="64">
+      <c r="G2" s="61">
         <v>11.57</v>
       </c>
-      <c r="H2" s="64">
+      <c r="H2" s="61">
         <v>182</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" s="62" t="s">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="59" t="s">
         <v>8</v>
       </c>
       <c r="B3" s="16">
@@ -10826,18 +10620,18 @@
       <c r="E3" s="16">
         <v>12.745000000000001</v>
       </c>
-      <c r="F3" s="64">
+      <c r="F3" s="61">
         <v>6.2</v>
       </c>
-      <c r="G3" s="64">
+      <c r="G3" s="61">
         <v>1.87</v>
       </c>
-      <c r="H3" s="64">
+      <c r="H3" s="61">
         <v>82</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" s="62" t="s">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="59" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="16">
@@ -10852,18 +10646,18 @@
       <c r="E4" s="16">
         <v>11.385</v>
       </c>
-      <c r="F4" s="64">
+      <c r="F4" s="61">
         <v>8.31</v>
       </c>
-      <c r="G4" s="64">
+      <c r="G4" s="61">
         <v>0.55000000000000004</v>
       </c>
-      <c r="H4" s="64">
+      <c r="H4" s="61">
         <v>52.43</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5" s="62" t="s">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="59" t="s">
         <v>25</v>
       </c>
       <c r="B5" s="16">
@@ -10878,13 +10672,13 @@
       <c r="E5" s="16">
         <v>7.8149999999999995</v>
       </c>
-      <c r="F5" s="64">
+      <c r="F5" s="61">
         <v>6.1099999999999994</v>
       </c>
-      <c r="G5" s="64">
+      <c r="G5" s="61">
         <v>1.83</v>
       </c>
-      <c r="H5" s="64">
+      <c r="H5" s="61">
         <v>27.71</v>
       </c>
     </row>

</xml_diff>